<commit_message>
Send reminders at 30/7/1 days before expiry
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2275C157-D38E-4AF4-8362-8A118A3F0977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC56A75A-CE44-4AB7-B878-35FEE0FDE95B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37035" yWindow="2820" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34455" yWindow="2010" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="clients" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="47">
   <si>
     <t>INDIVIDUAL/COMPANY</t>
   </si>
@@ -79,15 +79,6 @@
     <t>Domain renewal</t>
   </si>
   <si>
-    <t>Kevin Lim</t>
-  </si>
-  <si>
-    <t>016-5551234</t>
-  </si>
-  <si>
-    <t>Backup subscription renewal (not in window)</t>
-  </si>
-  <si>
     <t>Nur Izzah</t>
   </si>
   <si>
@@ -161,6 +152,15 @@
   </si>
   <si>
     <t xml:space="preserve">Arif </t>
+  </si>
+  <si>
+    <t>Iskhandar Shah</t>
+  </si>
+  <si>
+    <t>Antivirus License Renewal</t>
+  </si>
+  <si>
+    <t>013-6385897</t>
   </si>
 </sst>
 </file>
@@ -632,13 +632,13 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="J1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -648,9 +648,7 @@
       <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>44</v>
-      </c>
+      <c r="C2" s="3"/>
       <c r="D2" t="s">
         <v>9</v>
       </c>
@@ -672,7 +670,7 @@
         <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D3" t="s">
         <v>14</v>
@@ -692,11 +690,9 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>45</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="C4" s="3"/>
       <c r="D4" t="s">
         <v>17</v>
       </c>
@@ -715,20 +711,20 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="E5" s="2">
-        <v>46129</v>
+        <v>46114</v>
       </c>
       <c r="F5" t="s">
         <v>15</v>
       </c>
       <c r="G5" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -736,22 +732,22 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E6" s="2">
-        <v>46096</v>
+        <v>46114</v>
       </c>
       <c r="F6" t="s">
         <v>15</v>
       </c>
       <c r="G6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -759,17 +755,17 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F7" t="s">
         <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -777,11 +773,11 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E8" s="2">
         <v>46082</v>
@@ -790,7 +786,7 @@
         <v>15</v>
       </c>
       <c r="G8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -798,11 +794,11 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E9" s="2">
         <v>46085</v>
@@ -811,7 +807,7 @@
         <v>15</v>
       </c>
       <c r="G9" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -819,11 +815,11 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E10" s="2">
         <v>46109</v>
@@ -832,7 +828,7 @@
         <v>10</v>
       </c>
       <c r="G10" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -840,35 +836,33 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F11" t="s">
         <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" xr:uid="{91E34CC4-D4F1-4D66-B6BD-178D639EE306}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{A954686B-F1E4-461A-B06E-8E5E011612B3}"/>
-    <hyperlink ref="C2" r:id="rId3" xr:uid="{7B1EA981-B630-48F3-8DA0-0D55459A6126}"/>
-    <hyperlink ref="C6" r:id="rId4" xr:uid="{9FA2FA98-792F-424A-A83C-D75249276515}"/>
+    <hyperlink ref="C3" r:id="rId1" xr:uid="{A954686B-F1E4-461A-B06E-8E5E011612B3}"/>
+    <hyperlink ref="C6" r:id="rId2" xr:uid="{9FA2FA98-792F-424A-A83C-D75249276515}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="3">
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
-    <tablePart r:id="rId6"/>
-    <tablePart r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Excel for alignment
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E62896C-A7A6-458F-83DA-9CDF13B79E43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DB2DDC0-5335-4853-BD99-42826B6067B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36000" yWindow="2640" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="clients" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="62">
   <si>
     <t>INDIVIDUAL/COMPANY</t>
   </si>
@@ -43,9 +43,6 @@
     <t>REMARK</t>
   </si>
   <si>
-    <t>iamarifdanial@gmail.com</t>
-  </si>
-  <si>
     <t>Majlis Bandaraya Petaling Jaya</t>
   </si>
   <si>
@@ -116,6 +113,42 @@
   </si>
   <si>
     <t>MR. WONG CHIN WEI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">norelyani@mpag.gov.my </t>
+  </si>
+  <si>
+    <t>khairulnizam@mpj.gov.my</t>
+  </si>
+  <si>
+    <t>rahimi@mdpt.gov.my</t>
+  </si>
+  <si>
+    <t>ridhwan@mdsb.gov.my</t>
+  </si>
+  <si>
+    <t>zawani@mbas.gov.my</t>
+  </si>
+  <si>
+    <t>norhayati@jpbdselangor.gov.my</t>
+  </si>
+  <si>
+    <t>dominic@psterminal.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rahman@pspipeline.com.my </t>
+  </si>
+  <si>
+    <t>zam@mpjasin.gov.my</t>
+  </si>
+  <si>
+    <t>kunornadia@yahoo.com</t>
+  </si>
+  <si>
+    <t>damis@psterminal.com</t>
+  </si>
+  <si>
+    <t>cwwong@schmidtbmt.com</t>
   </si>
   <si>
     <t>019-2161005</t>
@@ -259,26 +292,33 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="5">
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -297,15 +337,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{91D90257-CA43-4392-B613-4DD09F72E19B}" name="Table1" displayName="Table1" ref="A1:G14" totalsRowShown="0">
   <autoFilter ref="A1:G14" xr:uid="{91D90257-CA43-4392-B613-4DD09F72E19B}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D2C5F103-82AA-4304-82E2-7181BC947C97}" name="INDIVIDUAL/COMPANY" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{1F830146-8D64-4B4D-BE03-1B25BE2530F7}" name="OFFICER NAME/NAME"/>
+    <tableColumn id="1" xr3:uid="{D2C5F103-82AA-4304-82E2-7181BC947C97}" name="INDIVIDUAL/COMPANY" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{1F830146-8D64-4B4D-BE03-1B25BE2530F7}" name="OFFICER NAME/NAME" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{E0AC4383-3583-457C-B06D-D72E355BA3DB}" name="EMAIL"/>
-    <tableColumn id="4" xr3:uid="{703A4075-CEFB-47AF-8378-880B0473CD44}" name="NO TEL" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{703A4075-CEFB-47AF-8378-880B0473CD44}" name="NO TEL" dataDxfId="2"/>
     <tableColumn id="5" xr3:uid="{811B1247-93CE-4F19-8082-75917D9AA4AC}" name="EXPIRED DATE" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{8C4C331C-4B8E-444D-9B8B-CDAFAAE3DE6A}" name="PC / SVR"/>
+    <tableColumn id="6" xr3:uid="{8C4C331C-4B8E-444D-9B8B-CDAFAAE3DE6A}" name="PC / SVR" dataDxfId="0"/>
     <tableColumn id="7" xr3:uid="{D4DB6335-DCB3-42D2-BA53-91B0B8DFDFC6}" name="REMARK"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -631,268 +671,268 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="B2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>32</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>43</v>
       </c>
       <c r="E2" s="5">
         <v>46136</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>43</v>
+      <c r="F2" s="4" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>33</v>
+      <c r="A3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>44</v>
       </c>
       <c r="E3" s="5">
         <v>46172</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>44</v>
+      <c r="F3" s="4" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>34</v>
+      <c r="A4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>45</v>
       </c>
       <c r="E4" s="5">
         <v>46277</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>45</v>
+      <c r="F4" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>35</v>
+      <c r="C5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>46</v>
       </c>
       <c r="E5" s="5">
         <v>46246</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="4">
         <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>36</v>
+      <c r="A6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>47</v>
       </c>
       <c r="E6" s="5">
         <v>46059</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="4">
         <v>250</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>37</v>
+      <c r="A7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>48</v>
       </c>
       <c r="E7" s="5">
         <v>46078</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>46</v>
+      <c r="F7" s="4" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>38</v>
+      <c r="A8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>49</v>
       </c>
       <c r="E8" s="5">
         <v>45612</v>
       </c>
-      <c r="F8" s="3"/>
+      <c r="F8" s="4"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>39</v>
+      <c r="A9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>50</v>
       </c>
       <c r="E9" s="5">
         <v>46213</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>47</v>
+      <c r="F9" s="4" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>40</v>
+      <c r="A10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>51</v>
       </c>
       <c r="E10" s="5">
         <v>46313</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="4">
         <v>200</v>
       </c>
       <c r="G10" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="3">
+      <c r="A11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="4">
         <v>60192462270</v>
       </c>
       <c r="E11" s="5">
         <v>46359</v>
       </c>
-      <c r="F11" s="3"/>
+      <c r="F11" s="4"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="3" t="s">
+      <c r="A12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>41</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>52</v>
       </c>
       <c r="E12" s="5">
         <v>46372</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="4">
         <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="3" t="s">
+      <c r="A13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>42</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>53</v>
       </c>
       <c r="E13" s="5">
         <v>46377</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="4">
         <v>7</v>
       </c>
       <c r="G13" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="3" t="s">
+      <c r="A14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>42</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>53</v>
       </c>
       <c r="E14" s="5">
         <v>46377</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="4">
         <v>8</v>
       </c>
       <c r="G14" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update xlsx - Testing
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Intern\PROJECT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C39CEF5A-3E32-44EB-AA1E-9F70E18369F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE24F69-97FD-4EE5-A0C1-391757B8D8F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34470" yWindow="1920" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="clients" sheetId="1" r:id="rId1"/>
@@ -202,7 +202,7 @@
     <t>iamarifdanial@gmail.com</t>
   </si>
   <si>
-    <t>arif@kyrolsecuritylabs.com, iamarifdanial@gmail.com</t>
+    <t>arif@kyrolsecuritylabs.com, 2024933617@student.uitm.edu.my</t>
   </si>
 </sst>
 </file>
@@ -638,7 +638,7 @@
   <cols>
     <col min="1" max="1" width="41.28515625" customWidth="1"/>
     <col min="2" max="2" width="37.28515625" customWidth="1"/>
-    <col min="3" max="3" width="58.28515625" customWidth="1"/>
+    <col min="3" max="3" width="120" customWidth="1"/>
     <col min="4" max="4" width="20.42578125" customWidth="1"/>
     <col min="5" max="5" width="15.42578125" customWidth="1"/>
     <col min="6" max="6" width="10.5703125" customWidth="1"/>

</xml_diff>

<commit_message>
Add PSP-FORTI sheet and generalize per-sheet detail fields
Onboard PSP-FORTI: a sheet with three stacked mini-tables (PS Pipeline,
PS Terminal Bintulu, PS Terminal Tawau) that each repeat their own
header row. loader.py now finds every header occurrence per sheet and
treats each as its own block, instead of assuming one header per sheet.

Replace the single detail_label/detail_value field with an ordered
"details" list per sheet config, since Fortinet rows carry more info
(Quantity, S/N, Remarks) than AV/Sangfor rows (one field each). Email
templates in main.py render however many detail rows a sheet defines.

PSP-FORTI test rows point at iamarifdanial@gmail.com with original
END DATEs preserved (all outside the 30-day window, so no live send
yet). Also fixed date-cell number formatting on Sangfor/PSP-FORTI to
match the existing clients sheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -3,11 +3,12 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="clients" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Sangfor" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="PSP-FORTI" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -16,11 +17,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,12 +40,6 @@
       <family val="2"/>
       <b val="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="8"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -88,9 +84,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -104,8 +100,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1034,6 +1031,9 @@
   </sheetPr>
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17.28515625" bestFit="1" customWidth="1" min="5" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1098,14 +1098,570 @@
           <t>019-2161005</t>
         </is>
       </c>
-      <c r="E2" s="6" t="n">
-        <v>46241.39551538732</v>
-      </c>
-      <c r="F2" s="6" t="n">
+      <c r="E2" s="7" t="n">
+        <v>46466</v>
+      </c>
+      <c r="F2" s="7" t="n">
         <v>45556</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>PS PIPELINE FORTINET RENEWAL LIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>COMPANY NAME</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PERSON IN CHARGE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PHONE NO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>END DATE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>REMINDER</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>QUANTITY</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>S/N</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>REMARKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PS Pipeline Sdn Bhd (SERVER ROOM)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>iamarifdanial@gmail.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>019-2161005</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>46394</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>46363</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>FG200FT922902625</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>PRODUCT MODEL - FG200F</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PS Pipeline Sdn Bhd (SERVER ROOM)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>iamarifdanial@gmail.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>019-2161005</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>46394</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>46363</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>FG200FT922901062</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>PRODUCT MODEL - FG200F</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PS Pipeline Sdn Bhd (ER)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>iamarifdanial@gmail.com</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>019-2161005</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>46366</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>46336</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>FG100FTK21028198</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>PRODUCT MODEL - FG100F</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PSP MRPP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>iamarifdanial@gmail.com</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>019-2161005</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>46399</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>46368</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>FG100FTK21041508</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>PRODUCT MODEL - FG100F</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PSP PDPP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>iamarifdanial@gmail.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>019-2161005</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>46366</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>46336</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>FG100FTK21041399</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>PRODUCT MODEL - FG100F</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PSP KLIA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>iamarifdanial@gmail.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>019-2161005</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>46366</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>46336</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>FG100FTK21029200</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>PRODUCT MODEL - FG100F</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>*** DATE FORMAT : DD/MM/YYYY</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PS TERMINAL (BINTULU) FORTINET RENEWAL LIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>COMPANY NAME</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PERSON IN CHARGE</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PHONE NO</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>END DATE</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>REMINDER</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>QUANTITY</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>S/N</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>REMARKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PS Terminal Bintulu</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>EN. DOMINIC TANGGAI AK SAIT</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>iamarifdanial@gmail.com</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>014-8979502</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>46348</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>FG100FTK20045129</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>*** DATE FORMAT : DD/MM/YYYY</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PS TERMINAL (TAWAU) FORTINET RENEWAL LIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>COMPANY NAME</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PERSON IN CHARGE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>PHONE NO</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>END DATE</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>REMINDER</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>QUANTITY</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>S/N</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>REMARKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PS Terminal Tawau</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>EN. DAMIS TILIP</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>iamarifdanial@gmail.com</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>011-19551456</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>46250</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>FG100FTK21000874</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Part Number - FC-10-F100F-950-02-12</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Onboard PLAN SELANGOR-FORTI, MD MERSING-FORTI, MP JASIN-FORTI sheets
Same Fortinet column layout as PSP-FORTI, added via the existing
SHEET_CONFIGS pattern. Also fixes recipient-email splitting in main.py:
MD MERSING-FORTI has multiple addresses separated by "/" instead of
",", and the old comma-only split would have treated the whole cell as
one broken address. Now splits on comma, semicolon, or slash.

MP JASIN-FORTI's source row has no END DATE, so it's correctly skipped
by the existing missing-date handling until that field is filled in.
Test rows use iamarifdanial@gmail.com where requested; MP JASIN kept
its real contact email since no override was asked for and the blank
date means it can't fire anyway.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -9,6 +9,9 @@
     <sheet name="clients" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Sangfor" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="PSP-FORTI" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="PLAN SELANGOR-FORTI" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="MD MERSING-FORTI" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="MP JASIN-FORTI" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1452,8 +1455,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -1559,8 +1560,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -1661,6 +1660,348 @@
       <c r="J20" t="inlineStr">
         <is>
           <t>Part Number - FC-10-F100F-950-02-12</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>PLAN MALAYSIA @ SELANGOR FORTINET RENEWAL LIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>COMPANY NAME</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PERSON IN CHARGE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PHONE NO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>END DATE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>REMINDER</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>QUANTITY</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>S/N</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>REMARKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PLAN SELANGOR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PN. SITI NORHAYATI BINTI MOKTI</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>iamarifdanial@gmail.com</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>46255</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>45829</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>FG200ETK19919553</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>PRODUCT MODEL - FG200E</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>MAJLIS DAERAH MERSING FORTINET RENEWAL LIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>COMPANY NAME</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PERSON IN CHARGE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PHONE NO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>END DATE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>REMINDER</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>QUANTITY</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>S/N</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>REMARKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MD MERSING</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EN. ZULKIFLI / EN. YUSOF</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>iamarifdanial@gmail.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>07-798 1818</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>45932</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>45577</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>FG100FTK19007567</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>PRODUCT MODEL - FG100F</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>*** DATE FORMAT : DD/MM/YYYY</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>MAJLIS PERBANDARAN JASIN FORTINET RENEWAL LIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>COMPANY NAME</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PERSON IN CHARGE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PHONE NO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>END DATE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>REMINDER</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>QUANTITY</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>S/N</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>REMARKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MP Jasin</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EN. ZAMZUL HIZAM BIN ABU HASSAN</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>zam@mpjasin.gov.my</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>06-3333333 EXT 2238</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>PRODUCT MODEL - FG80F</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add .dockerignore, unify team email list, restructure IILM's EMAIL column
Add .dockerignore to keep .env (real SMTP secrets), .git, and other
local-only files out of built Docker images -- COPY . . in the
Dockerfile would otherwise bake secrets straight into the image.

Replace the client-specific EMAIL values on Sangfor, PSP-FORTI, PLAN
SELANGOR-FORTI, MD MERSING-FORTI, MP JASIN-FORTI, and M365 with the
same internal team distribution list already used on AV, so all sheets
notify the same team.

Restructure IILM to read email from a real per-row EMAIL column
instead of a hardcoded fixed_email in loader.py, and remove the now-
redundant footer note listing the notification addresses. This makes
IILM consistent with every other sheet: the spreadsheet itself is the
single source of truth for contact emails, editable directly in Excel
without needing a code change.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="510" yWindow="2925" windowWidth="21600" windowHeight="11295" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="AV" sheetId="1" state="visible" r:id="rId1"/>
@@ -22,29 +22,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -55,9 +42,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
@@ -71,24 +61,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -98,80 +88,46 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="00000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="00000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00000000"/>
-      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -279,7 +235,7 @@
     <ext cx="1333500" cy="409575"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -289,7 +245,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -312,7 +270,7 @@
     <ext cx="1333500" cy="409575"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -322,7 +280,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -345,7 +305,7 @@
     <ext cx="1333500" cy="409575"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -355,7 +315,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -378,7 +340,7 @@
     <ext cx="1333500" cy="409575"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -388,7 +350,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -411,7 +375,7 @@
     <ext cx="1333500" cy="409575"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -421,7 +385,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -444,7 +410,7 @@
     <ext cx="1333500" cy="409575"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -454,7 +420,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -477,7 +445,7 @@
     <ext cx="1333500" cy="409575"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -487,7 +455,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -510,7 +480,7 @@
     <ext cx="1333500" cy="409575"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -520,7 +490,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -839,482 +811,481 @@
   <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="31" customWidth="1" min="7" max="7"/>
-    <col width="30.28515625" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="11"/>
+    <col width="44" customWidth="1" style="8" min="1" max="1"/>
+    <col width="34" customWidth="1" style="8" min="2" max="2"/>
+    <col width="142" customWidth="1" style="8" min="3" max="3"/>
+    <col width="21" customWidth="1" style="8" min="4" max="5"/>
+    <col width="10" customWidth="1" style="8" min="6" max="6"/>
+    <col width="31" customWidth="1" style="8" min="7" max="7"/>
+    <col width="30.28515625" customWidth="1" style="8" min="8" max="8"/>
+    <col width="11" customWidth="1" style="8" min="9" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>INDIVIDUAL/COMPANY</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>OFFICER NAME/NAME</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>NO TEL</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EXPIRED DATE</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>PC / SVR</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>CUST EMAIL</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Majlis Bandaraya Petaling Jaya</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>EN. KHAIRUL NIZAM BIN AB JABAR</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>019-2161005</t>
         </is>
       </c>
-      <c r="E2" s="11" t="n">
+      <c r="E2" s="4" t="n">
         <v>46136</v>
       </c>
-      <c r="F2" s="9" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>1800/80</t>
         </is>
       </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>khairulnizam@mpj.gov.my</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Majlis Perbadanan Alor Gajah</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>PN NOR ELYANI BINTI RAMLI</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>017-6200053</t>
         </is>
       </c>
-      <c r="E3" s="11" t="n">
+      <c r="E3" s="4" t="n">
         <v>46172</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>85/15</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">norelyani@mpag.gov.my </t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Majlis Daerah Perak Tengah</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">EN. MOHAMAD RAHIMI BIN HAMIZI </t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>013-7992042</t>
         </is>
       </c>
-      <c r="E4" s="12" t="n">
+      <c r="E4" s="5" t="n">
         <v>46277</v>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>70/1</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>rahimi@mdpt.gov.my</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+    <row r="5" ht="30" customHeight="1" s="8">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Majlis Daerah Sabak Bernam</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">EN. MUHAMMAD RIDHWAN BIN IKHSAN </t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>012-2686094</t>
         </is>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="5" t="n">
         <v>46246</v>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F5" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>ridhwan@mdsb.gov.my</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Majlis Bandaraya Alor Setar</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EN. NOORZAWANI BIN JUSOH</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>04-7301255</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="4" t="n">
         <v>46059</v>
       </c>
-      <c r="F6" s="9" t="n">
+      <c r="F6" s="2" t="n">
         <v>250</v>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>zawani@mbas.gov.my</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Jabatan Perancangan Bandar &amp; Desa Selangor</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>PN. SITI NORHAYATI BINTI MOKTI</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>603 5511 6666</t>
         </is>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="4" t="n">
         <v>46078</v>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>105/1</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>norhayati@jpbdselangor.gov.my</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>PS Terminal (Bintulu)</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EN. DOMINIC TANGGAI</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>08-6255442</t>
         </is>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="4" t="n">
         <v>45612</v>
       </c>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>dominic@psterminal.com</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>PS Pipeline (KVDT)</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>603-88943333</t>
         </is>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="5" t="n">
         <v>46213</v>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>54/1</t>
         </is>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">rahman@pspipeline.com.my </t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="10" ht="30" customHeight="1" s="8">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Majlis Perbandaran Jasin</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EN. ZAMZUL HIZAM BIN ABU HASSAN</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>06-3333333 EXT 2238</t>
         </is>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="5" t="n">
         <v>46313</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="F10" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>zam@mpjasin.gov.my</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>KYROL AV INDIVIDUAL</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>PN. KU NOR NADIA</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="n">
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
         <v>60192462270</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="5" t="n">
         <v>46359</v>
       </c>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>kunornadia@yahoo.com</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>PS Terminal (Tawau)</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EN.DAMIS TILIP</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>08-9776903</t>
         </is>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="5" t="n">
         <v>46372</v>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="F12" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="G12" s="10" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>damis@psterminal.com</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>SCHMIDT BIOMEDTECH</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>MR. WONG CHIN WEI</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>03-79577122</t>
         </is>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="5" t="n">
         <v>46377</v>
       </c>
-      <c r="F13" s="9" t="n">
+      <c r="F13" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G13" s="10" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>cwwong@schmidtbmt.com</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>SCHMIDT BIOMEDTECH</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>MR. WONG CHIN WEI</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>03-79577122</t>
         </is>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="5" t="n">
         <v>46377</v>
       </c>
-      <c r="F14" s="9" t="n">
+      <c r="F14" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="G14" s="10" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>cwwong@schmidtbmt.com</t>
         </is>
@@ -1366,89 +1337,88 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="21" bestFit="1" customWidth="1" min="5" max="6"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" style="8" min="1" max="1"/>
+    <col width="30" customWidth="1" style="8" min="2" max="2"/>
+    <col width="25" customWidth="1" style="8" min="3" max="3"/>
+    <col width="13" customWidth="1" style="8" min="4" max="4"/>
+    <col width="21" bestFit="1" customWidth="1" style="8" min="5" max="5"/>
+    <col width="21" customWidth="1" style="8" min="6" max="6"/>
+    <col width="10" customWidth="1" style="8" min="7" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="8">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>COMPANY NAME</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>PERSON IN CHARGE</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>PHONE NO</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>END DATE</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>REMINDER</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>QUANTITY</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+    <row r="2" ht="30" customHeight="1" s="8">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>PS Pipeline Sdn Bhd</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>019-2161005</t>
         </is>
       </c>
-      <c r="E2" s="13" t="n">
+      <c r="E2" s="5" t="n">
         <v>46466</v>
       </c>
-      <c r="F2" s="14" t="n">
+      <c r="F2" s="6" t="n">
         <v>45556</v>
       </c>
-      <c r="G2" s="9" t="n">
+      <c r="G2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="9" t="n"/>
+      <c r="H2" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1465,336 +1435,335 @@
   <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="37" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" style="8" min="1" max="1"/>
+    <col width="35" customWidth="1" style="8" min="2" max="2"/>
+    <col width="30" customWidth="1" style="8" min="3" max="3"/>
+    <col width="25" customWidth="1" style="8" min="4" max="4"/>
+    <col width="14" customWidth="1" style="8" min="5" max="5"/>
+    <col width="21" customWidth="1" style="8" min="6" max="7"/>
+    <col width="10" customWidth="1" style="8" min="8" max="8"/>
+    <col width="18" customWidth="1" style="8" min="9" max="9"/>
+    <col width="37" customWidth="1" style="8" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1" s="8">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>PS PIPELINE FORTINET RENEWAL LIST</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+    <row r="2" ht="30" customHeight="1" s="8">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>COMPANY NAME</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>PERSON IN CHARGE</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>PHONE NO</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>END DATE</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>REMINDER</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>QUANTITY</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>S/N</t>
         </is>
       </c>
-      <c r="J2" s="8" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="9" t="n">
+    <row r="3" ht="30" customHeight="1" s="8">
+      <c r="A3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>PS Pipeline Sdn Bhd (SERVER ROOM)</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>019-2161005</t>
         </is>
       </c>
-      <c r="F3" s="13" t="n">
+      <c r="F3" s="5" t="n">
         <v>46394</v>
       </c>
-      <c r="G3" s="14" t="n">
+      <c r="G3" s="6" t="n">
         <v>46363</v>
       </c>
-      <c r="H3" s="9" t="n">
+      <c r="H3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="9" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>FG200FT922902625</t>
         </is>
       </c>
-      <c r="J3" s="9" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>PRODUCT MODEL - FG200F</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="9" t="n">
+    <row r="4" ht="30" customHeight="1" s="8">
+      <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>PS Pipeline Sdn Bhd (SERVER ROOM)</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>019-2161005</t>
         </is>
       </c>
-      <c r="F4" s="13" t="n">
+      <c r="F4" s="5" t="n">
         <v>46394</v>
       </c>
-      <c r="G4" s="14" t="n">
+      <c r="G4" s="6" t="n">
         <v>46363</v>
       </c>
-      <c r="H4" s="9" t="n">
+      <c r="H4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>FG200FT922901062</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>PRODUCT MODEL - FG200F</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="9" t="n">
+    <row r="5" ht="30" customHeight="1" s="8">
+      <c r="A5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>PS Pipeline Sdn Bhd (ER)</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>019-2161005</t>
         </is>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="5" t="n">
         <v>46366</v>
       </c>
-      <c r="G5" s="14" t="n">
+      <c r="G5" s="6" t="n">
         <v>46336</v>
       </c>
-      <c r="H5" s="9" t="n">
+      <c r="H5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="9" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>FG100FTK21028198</t>
         </is>
       </c>
-      <c r="J5" s="9" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>PRODUCT MODEL - FG100F</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="9" t="n">
+    <row r="6" ht="30" customHeight="1" s="8">
+      <c r="A6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>PSP MRPP</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>019-2161005</t>
         </is>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="5" t="n">
         <v>46399</v>
       </c>
-      <c r="G6" s="14" t="n">
+      <c r="G6" s="6" t="n">
         <v>46368</v>
       </c>
-      <c r="H6" s="9" t="n">
+      <c r="H6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I6" s="9" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>FG100FTK21041508</t>
         </is>
       </c>
-      <c r="J6" s="9" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>PRODUCT MODEL - FG100F</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="9" t="n">
+    <row r="7" ht="30" customHeight="1" s="8">
+      <c r="A7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>PSP PDPP</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>019-2161005</t>
         </is>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="5" t="n">
         <v>46366</v>
       </c>
-      <c r="G7" s="14" t="n">
+      <c r="G7" s="6" t="n">
         <v>46336</v>
       </c>
-      <c r="H7" s="9" t="n">
+      <c r="H7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="9" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>FG100FTK21041399</t>
         </is>
       </c>
-      <c r="J7" s="9" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>PRODUCT MODEL - FG100F</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="9" t="n">
+    <row r="8" ht="30" customHeight="1" s="8">
+      <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>PSP KLIA</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>EN. ABDUL RAHMAN BIN ZAKARIA</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>019-2161005</t>
         </is>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="5" t="n">
         <v>46366</v>
       </c>
-      <c r="G8" s="14" t="n">
+      <c r="G8" s="6" t="n">
         <v>46336</v>
       </c>
-      <c r="H8" s="9" t="n">
+      <c r="H8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>FG100FTK21029200</t>
         </is>
       </c>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>PRODUCT MODEL - FG100F</t>
         </is>
@@ -1807,104 +1776,104 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+    <row r="12" ht="15.75" customHeight="1" s="8">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>PS TERMINAL (BINTULU) FORTINET RENEWAL LIST</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="13" ht="30" customHeight="1" s="8">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>COMPANY NAME</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>PERSON IN CHARGE</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>EMAIL</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>PHONE NO</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>END DATE</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
+      <c r="G13" s="1" t="inlineStr">
         <is>
           <t>REMINDER</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="H13" s="1" t="inlineStr">
         <is>
           <t>QUANTITY</t>
         </is>
       </c>
-      <c r="I13" s="8" t="inlineStr">
+      <c r="I13" s="1" t="inlineStr">
         <is>
           <t>S/N</t>
         </is>
       </c>
-      <c r="J13" s="8" t="inlineStr">
+      <c r="J13" s="1" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="n">
+      <c r="A14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>PS Terminal Bintulu</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>EN. DOMINIC TANGGAI AK SAIT</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>014-8979502</t>
         </is>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="5" t="n">
         <v>46348</v>
       </c>
-      <c r="G14" s="14" t="n">
+      <c r="G14" s="6" t="n">
         <v>46317</v>
       </c>
-      <c r="H14" s="9" t="n">
+      <c r="H14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I14" s="9" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>FG100FTK20045129</t>
         </is>
       </c>
-      <c r="J14" s="9" t="n"/>
+      <c r="J14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1913,104 +1882,104 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+    <row r="18" ht="15.75" customHeight="1" s="8">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>PS TERMINAL (TAWAU) FORTINET RENEWAL LIST</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="19" ht="30" customHeight="1" s="8">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>COMPANY NAME</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>PERSON IN CHARGE</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>EMAIL</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>PHONE NO</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>END DATE</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
+      <c r="G19" s="1" t="inlineStr">
         <is>
           <t>REMINDER</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="H19" s="1" t="inlineStr">
         <is>
           <t>QUANTITY</t>
         </is>
       </c>
-      <c r="I19" s="8" t="inlineStr">
+      <c r="I19" s="1" t="inlineStr">
         <is>
           <t>S/N</t>
         </is>
       </c>
-      <c r="J19" s="8" t="inlineStr">
+      <c r="J19" s="1" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="n">
+      <c r="A20" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>PS Terminal Tawau</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>EN. DAMIS TILIP</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>011-19551456</t>
         </is>
       </c>
-      <c r="F20" s="13" t="n">
+      <c r="F20" s="5" t="n">
         <v>46313</v>
       </c>
-      <c r="G20" s="14" t="n">
+      <c r="G20" s="6" t="n">
         <v>46250</v>
       </c>
-      <c r="H20" s="9" t="n">
+      <c r="H20" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I20" s="9" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>FG100FTK21000874</t>
         </is>
       </c>
-      <c r="J20" s="9" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Part Number - FC-10-F100F-950-02-12</t>
         </is>
@@ -2036,112 +2005,111 @@
   <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" style="8" min="1" max="1"/>
+    <col width="15" customWidth="1" style="8" min="2" max="2"/>
+    <col width="32" customWidth="1" style="8" min="3" max="3"/>
+    <col width="25" customWidth="1" style="8" min="4" max="4"/>
+    <col width="10" customWidth="1" style="8" min="5" max="5"/>
+    <col width="21" customWidth="1" style="8" min="6" max="7"/>
+    <col width="10" customWidth="1" style="8" min="8" max="8"/>
+    <col width="18" customWidth="1" style="8" min="9" max="9"/>
+    <col width="24" customWidth="1" style="8" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1" s="8">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>PLAN MALAYSIA @ SELANGOR FORTINET RENEWAL LIST</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+    <row r="2" ht="30" customHeight="1" s="8">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>COMPANY NAME</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>PERSON IN CHARGE</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>PHONE NO</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>END DATE</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>REMINDER</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>QUANTITY</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>S/N</t>
         </is>
       </c>
-      <c r="J2" s="8" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="9" t="n">
+    <row r="3" ht="30" customHeight="1" s="8">
+      <c r="A3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>PLAN SELANGOR</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>PN. SITI NORHAYATI BINTI MOKTI</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="n"/>
-      <c r="F3" s="13" t="n">
-        <v>46241.50735334491</v>
-      </c>
-      <c r="G3" s="14" t="n">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="5" t="n">
+        <v>46255</v>
+      </c>
+      <c r="G3" s="6" t="n">
         <v>45829</v>
       </c>
-      <c r="H3" s="9" t="n">
+      <c r="H3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="9" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>FG200ETK19919553</t>
         </is>
       </c>
-      <c r="J3" s="9" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>PRODUCT MODEL - FG200E</t>
         </is>
@@ -2165,116 +2133,115 @@
   <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" style="8" min="1" max="1"/>
+    <col width="14" customWidth="1" style="8" min="2" max="2"/>
+    <col width="26" customWidth="1" style="8" min="3" max="3"/>
+    <col width="25" customWidth="1" style="8" min="4" max="4"/>
+    <col width="13" customWidth="1" style="8" min="5" max="5"/>
+    <col width="21" customWidth="1" style="8" min="6" max="7"/>
+    <col width="10" customWidth="1" style="8" min="8" max="8"/>
+    <col width="18" customWidth="1" style="8" min="9" max="9"/>
+    <col width="24" customWidth="1" style="8" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1" s="8">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>MAJLIS DAERAH MERSING FORTINET RENEWAL LIST</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+    <row r="2" ht="30" customHeight="1" s="8">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>COMPANY NAME</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>PERSON IN CHARGE</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>PHONE NO</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>END DATE</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>REMINDER</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>QUANTITY</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>S/N</t>
         </is>
       </c>
-      <c r="J2" s="8" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="9" t="n">
+    <row r="3" ht="30" customHeight="1" s="8">
+      <c r="A3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>MD MERSING</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>EN. ZULKIFLI / EN. YUSOF</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>07-798 1818</t>
         </is>
       </c>
-      <c r="F3" s="16" t="n">
+      <c r="F3" s="4" t="n">
         <v>45932</v>
       </c>
-      <c r="G3" s="14" t="n">
+      <c r="G3" s="6" t="n">
         <v>45577</v>
       </c>
-      <c r="H3" s="9" t="n">
+      <c r="H3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="9" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>FG100FTK19007567</t>
         </is>
       </c>
-      <c r="J3" s="9" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>PRODUCT MODEL - FG100F</t>
         </is>
@@ -2305,108 +2272,105 @@
   <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" style="8" min="1" max="1"/>
+    <col width="14" customWidth="1" style="8" min="2" max="2"/>
+    <col width="33" customWidth="1" style="8" min="3" max="3"/>
+    <col width="20" customWidth="1" style="8" min="4" max="4"/>
+    <col width="21" customWidth="1" style="8" min="5" max="5"/>
+    <col width="10" customWidth="1" style="8" min="6" max="9"/>
+    <col width="23" customWidth="1" style="8" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1" s="8">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>MAJLIS PERBANDARAN JASIN FORTINET RENEWAL LIST</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+    <row r="2" ht="30" customHeight="1" s="8">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>COMPANY NAME</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>PERSON IN CHARGE</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>PHONE NO</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>END DATE</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>REMINDER</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>QUANTITY</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>S/N</t>
         </is>
       </c>
-      <c r="J2" s="8" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="9" t="n">
+    <row r="3" ht="30" customHeight="1" s="8">
+      <c r="A3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>MP Jasin</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>EN. ZAMZUL HIZAM BIN ABU HASSAN</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>06-3333333 EXT 2238</t>
         </is>
       </c>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="9" t="n"/>
-      <c r="H3" s="9" t="n">
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="9" t="n"/>
-      <c r="J3" s="9" t="inlineStr">
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>PRODUCT MODEL - FG80F</t>
         </is>
@@ -2427,383 +2391,403 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" style="8" min="1" max="1"/>
+    <col width="10" customWidth="1" style="8" min="2" max="2"/>
+    <col width="45" customWidth="1" style="8" min="3" max="3"/>
+    <col width="32" customWidth="1" style="8" min="4" max="4"/>
+    <col width="21" customWidth="1" style="8" min="5" max="6"/>
+    <col width="11" customWidth="1" style="8" min="7" max="7"/>
+    <col width="45" customWidth="1" style="8" min="8" max="8"/>
+    <col width="10" customWidth="1" style="8" min="9" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1" s="8">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>IILM'S RENEWAL LIST</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>BRAND</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>PRODUCT</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>LICENSE NUMBER</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>END DATE</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>REMINDER</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>QUANTITY</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>S/N</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="J2" s="8" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="9" t="n">
+    <row r="3" ht="30" customHeight="1" s="8">
+      <c r="A3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>SOPHOS</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Central Intercept X Advanced (SKU: CIXA0U12ACRCAA Old SKU: )</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>L0006655661</t>
         </is>
       </c>
-      <c r="E3" s="13" t="n">
+      <c r="E3" s="5" t="n">
         <v>46296</v>
       </c>
-      <c r="F3" s="14" t="n">
+      <c r="F3" s="6" t="n">
         <v>45870</v>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>35 USERS</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr"/>
-      <c r="I3" s="9" t="inlineStr"/>
-      <c r="J3" s="9" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="n">
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1" s="8">
+      <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>SOPHOS</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Central Intercept X Advanced for Server (SKU: CIXA0S12BARCAA Old SKU: )</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>L0005748816</t>
         </is>
       </c>
-      <c r="E4" s="13" t="n">
+      <c r="E4" s="5" t="n">
         <v>46296</v>
       </c>
-      <c r="F4" s="14" t="n">
+      <c r="F4" s="6" t="n">
         <v>45870</v>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>6 SERVERS</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr"/>
-      <c r="I4" s="9" t="inlineStr"/>
-      <c r="J4" s="9" t="inlineStr"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>PEPLINK</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Peplink BPL-305</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>1825-D3C8-D97A, 1825-D3D8-C87B</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="5" t="n">
         <v>46342</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="6" t="n">
         <v>46281</v>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="G5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>1825-D3C8-D97A, 1825-D3D8-C87B</t>
         </is>
       </c>
-      <c r="I5" s="9" t="inlineStr"/>
-      <c r="J5" s="9" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n">
+      <c r="A6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>FORTINET</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>FortiGate-100F</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>FC-10-F100F-950-02-12</t>
         </is>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="5" t="n">
         <v>46308</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="6" t="n">
         <v>46278</v>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="9" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>FG100FTK20035388</t>
         </is>
       </c>
-      <c r="I6" s="9" t="inlineStr"/>
-      <c r="J6" s="9" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n">
+      <c r="A7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>FORTINET</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>FortiGate-100F</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>FC-10-F100F-950-02-12</t>
         </is>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="5" t="n">
         <v>46308</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="6" t="n">
         <v>46278</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>FG100FTK20036888</t>
         </is>
       </c>
-      <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="9" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="n">
+      <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>FORTINET</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>FortiMail Cloud</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>FC1-10-FECLD-423-02-12</t>
         </is>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="5" t="n">
         <v>46308</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="6" t="n">
         <v>46278</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="9" t="inlineStr"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n">
+      <c r="A9" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>CISCO</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>C9200L-24-4X-E</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>206939165</t>
         </is>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="5" t="n">
         <v>46381</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="6" t="n">
         <v>44190</v>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="9" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>FVH29342AM9</t>
         </is>
       </c>
-      <c r="I9" s="9" t="inlineStr"/>
-      <c r="J9" s="9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="n">
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1" s="8">
+      <c r="A10" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>FORTINET</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Fortiguard &amp; Client</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr"/>
-      <c r="E10" s="13" t="n">
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="5" t="n">
         <v>46311</v>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="6" t="n">
         <v>46281</v>
       </c>
-      <c r="G10" s="9" t="n">
+      <c r="G10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H10" s="9" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>FCTEMS8823003672, FCTEMS8822001697, FCTEMS8822201698</t>
         </is>
       </c>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="9" t="inlineStr"/>
-    </row>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n"/>
+    </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr"/>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>** EMAIL</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="9" t="n"/>
-      <c r="H13" s="9" t="n"/>
-      <c r="I13" s="9" t="n"/>
-      <c r="J13" s="9" t="n"/>
-    </row>
-    <row r="14">
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-    </row>
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+    </row>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -2822,163 +2806,161 @@
   <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" style="8" min="1" max="1"/>
+    <col width="23" customWidth="1" style="8" min="2" max="2"/>
+    <col width="18" customWidth="1" style="8" min="3" max="3"/>
+    <col width="31" customWidth="1" style="8" min="4" max="4"/>
+    <col width="15" customWidth="1" style="8" min="5" max="5"/>
+    <col width="21" customWidth="1" style="8" min="6" max="6"/>
+    <col width="10" customWidth="1" style="8" min="7" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+    <row r="1" ht="15.75" customHeight="1" s="8">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>CLIENT'S M365 RENEWAL LIST</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+    <row r="2" ht="30" customHeight="1" s="8">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>COMPANY NAME</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>PERSON IN CHARGE</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>PHONE NO</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>END DATE</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>REMINDER</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>QUANTITY</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="9" t="n">
+    <row r="3" ht="30" customHeight="1" s="8">
+      <c r="A3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>PLANMALAYSIA@Selangor</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>PN.SITI</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>603 5511 6666</t>
         </is>
       </c>
-      <c r="F3" s="16" t="n">
+      <c r="F3" s="4" t="n">
         <v>45993</v>
       </c>
-      <c r="G3" s="9" t="n"/>
-      <c r="H3" s="9" t="n"/>
-      <c r="I3" s="9" t="inlineStr"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="n">
+      <c r="A4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>ILS Offshore Sdn Bhd</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>EN FADHLI</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr"/>
-      <c r="F4" s="16" t="n">
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="4" t="n">
         <v>45723</v>
       </c>
-      <c r="G4" s="9" t="n"/>
-      <c r="H4" s="9" t="n">
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I4" s="9" t="inlineStr"/>
+      <c r="I4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Kaysix Sdn Bhd</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>NURUL SYAFINAZ</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>iamarifdanial@gmail.com</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>iskhandar@kyrolsecuritylabs.com, syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>019-649 1913</t>
         </is>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="4" t="n">
         <v>45737</v>
       </c>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="9" t="n">
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="I5" s="9" t="inlineStr"/>
+      <c r="I5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">

</xml_diff>

<commit_message>
Style License Pentest/SOC sheets to match other sheets (table + logo)
Restructure the two new license sheets into a proper formatted table
matching the existing sheets: merged title row, yellow bold header with
thin borders, bordered/centered data cells, DD/MM/YYYY date format,
fitted column widths, and the Kyrol logo anchored top-right.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,8 +54,18 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF808080"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -80,8 +90,18 @@
         <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -104,12 +124,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -133,6 +167,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -253,6 +300,39 @@
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7820025" cy="2419350"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
         <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
@@ -498,6 +578,39 @@
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7820025" cy="2419350"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
         <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1341,73 +1454,84 @@
   </sheetPr>
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="8" min="1" max="1"/>
+    <col width="26" customWidth="1" style="8" min="2" max="2"/>
+    <col width="50" customWidth="1" style="8" min="3" max="3"/>
+    <col width="16" customWidth="1" style="8" min="4" max="4"/>
+    <col width="34" customWidth="1" style="8" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="20" customHeight="1" s="8">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>KYROL SECURITY LABS - SOC LICENSE RENEWAL LIST</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="30" customHeight="1" s="8">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>COMPANY NAME</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>EXPIRY DATE</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" ht="75" customHeight="1" s="8">
+      <c r="A3" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Kyrol Security Labs</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com, adawiyah@kyrolsecuritylabs.com</t>
         </is>
       </c>
-      <c r="D3" s="10" t="n">
+      <c r="D3" s="13" t="n">
         <v>46358</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>SOC license renewal</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>*** DATE FORMAT : DD/MM/YYYY</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3064,72 +3188,83 @@
   </sheetPr>
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="8" min="1" max="1"/>
+    <col width="26" customWidth="1" style="8" min="2" max="2"/>
+    <col width="50" customWidth="1" style="8" min="3" max="3"/>
+    <col width="16" customWidth="1" style="8" min="4" max="4"/>
+    <col width="34" customWidth="1" style="8" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="20" customHeight="1" s="8">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>KYROL SECURITY LABS - PENTEST LICENSE RENEWAL LIST</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="30" customHeight="1" s="8">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>COMPANY NAME</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>EXPIRY DATE</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" ht="75" customHeight="1" s="8">
+      <c r="A3" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Kyrol Security Labs</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>syafinaz.rosli@kyrolsecuritylabs.com, khairol@kyrolsecuritylabs.com, elle@kyrolsecuritylabs.com, adawiyah@kyrolsecuritylabs.com</t>
         </is>
       </c>
-      <c r="D3" s="10" t="n">
+      <c r="D3" s="13" t="n">
         <v>46582</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>Penetration testing license renewal</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>*** DATE FORMAT : DD/MM/YYYY</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
change date format on clients.xlsx and update demo email
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\email-reminder\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD2D0518-59B6-4197-9089-4B6B4CD0DA5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABCFEF41-9B24-4432-84B5-DDC4976FCD8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AV" sheetId="1" r:id="rId1"/>
@@ -67,9 +67,6 @@
     <t>1800/80</t>
   </si>
   <si>
-    <t>khairulnizam@mpj.gov.my</t>
-  </si>
-  <si>
     <t>Majlis Perbadanan Alor Gajah</t>
   </si>
   <si>
@@ -479,6 +476,9 @@
   </si>
   <si>
     <t>SOC license renewal</t>
+  </si>
+  <si>
+    <t>mrozi@mpj.gov.my</t>
   </si>
 </sst>
 </file>
@@ -487,7 +487,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="166" formatCode="[$-14809]d/m/yyyy;@"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -600,7 +600,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -609,29 +609,34 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -642,7 +647,7 @@
       <alignment horizontal="left" vertical="bottom"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+      <numFmt numFmtId="166" formatCode="[$-14809]d/m/yyyy;@"/>
       <alignment horizontal="left" vertical="bottom"/>
     </dxf>
     <dxf>
@@ -1386,7 +1391,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
@@ -1412,7 +1417,7 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -1435,204 +1440,204 @@
       <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="10">
         <v>46136</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>12</v>
+      <c r="G2" s="14" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="11">
+        <v>46543</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="4">
-        <v>46172</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="11">
+        <v>46277</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="5">
-        <v>46277</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="30" customHeight="1">
       <c r="A5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="5">
+      <c r="E5" s="11">
         <v>46364</v>
       </c>
       <c r="F5" s="2">
         <v>150</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="4">
-        <v>46059</v>
+      <c r="E6" s="10">
+        <v>46175</v>
       </c>
       <c r="F6" s="2">
         <v>250</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="11">
+        <v>46513</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="4">
-        <v>46078</v>
-      </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E8" s="4">
-        <v>45612</v>
+      <c r="E8" s="10">
+        <v>46142</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="11">
+        <v>46302</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="5">
-        <v>46213</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="3" t="s">
         <v>43</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="30" customHeight="1">
       <c r="A10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" s="5">
+      <c r="E10" s="11">
         <v>46313</v>
       </c>
       <c r="F10" s="2">
         <v>200</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>9</v>
@@ -1640,82 +1645,85 @@
       <c r="D11" s="2">
         <v>60192462270</v>
       </c>
-      <c r="E11" s="5">
-        <v>46359</v>
+      <c r="E11" s="11">
+        <v>46726</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E12" s="5">
-        <v>46372</v>
+      <c r="E12" s="11">
+        <v>46723</v>
       </c>
       <c r="F12" s="2">
         <v>14</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E13" s="5">
+      <c r="E13" s="11">
         <v>46377</v>
       </c>
       <c r="F13" s="2">
         <v>7</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" s="5">
+      <c r="E14" s="11">
         <v>46377</v>
       </c>
       <c r="F14" s="2">
         <v>8</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>59</v>
-      </c>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="E15" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1726,30 +1734,31 @@
     <hyperlink ref="C4" r:id="rId5" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
     <hyperlink ref="G4" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="C5" r:id="rId7" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="G5" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="C6" r:id="rId9" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="G6" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="C7" r:id="rId11" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="G7" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="C8" r:id="rId13" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="G8" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="C9" r:id="rId15" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="G9" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="C10" r:id="rId17" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="G10" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="C11" r:id="rId19" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="G11" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="C12" r:id="rId21" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="G12" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="C13" r:id="rId23" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="G13" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="C14" r:id="rId25" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="G14" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="C6" r:id="rId8" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="G6" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="C7" r:id="rId10" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="G7" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="C8" r:id="rId12" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="G8" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="C9" r:id="rId14" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="G9" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="C10" r:id="rId16" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="G10" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="C11" r:id="rId18" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="G11" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="C12" r:id="rId20" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="G12" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="C13" r:id="rId22" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="G13" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="C14" r:id="rId24" display="iskhandar@kyrolsecuritylabs.com" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="G14" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="G5" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId27"/>
+  <pageSetup orientation="portrait" r:id="rId27"/>
+  <drawing r:id="rId28"/>
   <tableParts count="1">
-    <tablePart r:id="rId28"/>
+    <tablePart r:id="rId29"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1767,51 +1776,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+    </row>
+    <row r="2" spans="1:5" ht="30" customHeight="1">
+      <c r="A2" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="75" customHeight="1">
+      <c r="A3" s="5">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D3" s="15">
+        <v>46358</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-    </row>
-    <row r="2" spans="1:5" ht="30" customHeight="1">
-      <c r="A2" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="75" customHeight="1">
-      <c r="A3" s="7">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="D3" s="8">
-        <v>46358</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>149</v>
-      </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="9" t="s">
-        <v>84</v>
+      <c r="A4" s="6" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1839,36 +1848,36 @@
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
@@ -1876,10 +1885,10 @@
       <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="11">
         <v>46466</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="4">
         <v>45556</v>
       </c>
       <c r="G2" s="2">
@@ -1910,49 +1919,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A1" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
+      <c r="A1" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1">
@@ -1960,10 +1969,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>9</v>
@@ -1971,20 +1980,20 @@
       <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="11">
         <v>46394</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="4">
         <v>46363</v>
       </c>
       <c r="H3" s="2">
         <v>1</v>
       </c>
       <c r="I3" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1">
@@ -1992,10 +2001,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>9</v>
@@ -2003,20 +2012,20 @@
       <c r="E4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="11">
         <v>46394</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="4">
         <v>46363</v>
       </c>
       <c r="H4" s="2">
         <v>1</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1">
@@ -2024,10 +2033,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>9</v>
@@ -2035,20 +2044,20 @@
       <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="11">
         <v>46366</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="4">
         <v>46336</v>
       </c>
       <c r="H5" s="2">
         <v>1</v>
       </c>
       <c r="I5" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="30" customHeight="1">
@@ -2056,10 +2065,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>9</v>
@@ -2067,20 +2076,20 @@
       <c r="E6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="11">
         <v>46399</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="4">
         <v>46368</v>
       </c>
       <c r="H6" s="2">
         <v>1</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="30" customHeight="1">
@@ -2088,10 +2097,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>9</v>
@@ -2099,20 +2108,20 @@
       <c r="E7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="11">
         <v>46366</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="4">
         <v>46336</v>
       </c>
       <c r="H7" s="2">
         <v>1</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="30" customHeight="1">
@@ -2120,10 +2129,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>9</v>
@@ -2131,71 +2140,71 @@
       <c r="E8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="11">
         <v>46366</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="4">
         <v>46336</v>
       </c>
       <c r="H8" s="2">
         <v>1</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" customHeight="1">
+      <c r="A12" s="12" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A12" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
     </row>
     <row r="13" spans="1:10" ht="30" customHeight="1">
       <c r="A13" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="120" customHeight="1">
@@ -2203,80 +2212,80 @@
         <v>1</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F14" s="5">
+      <c r="F14" s="11">
         <v>46348</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G14" s="4">
         <v>46317</v>
       </c>
       <c r="H14" s="2">
         <v>1</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A18" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
+      <c r="A18" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
     </row>
     <row r="19" spans="1:10" ht="30" customHeight="1">
       <c r="A19" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I19" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H19" s="1" t="s">
+      <c r="J19" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="120" customHeight="1">
@@ -2284,31 +2293,31 @@
         <v>1</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F20" s="5">
+      <c r="F20" s="11">
         <v>46313</v>
       </c>
-      <c r="G20" s="6">
+      <c r="G20" s="4">
         <v>46250</v>
       </c>
       <c r="H20" s="2">
         <v>1</v>
       </c>
       <c r="I20" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="J20" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -2339,49 +2348,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A1" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
+      <c r="A1" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1">
@@ -2389,29 +2398,29 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="2"/>
-      <c r="F3" s="5">
+      <c r="F3" s="11">
         <v>46255</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="4">
         <v>45829</v>
       </c>
       <c r="H3" s="2">
         <v>1</v>
       </c>
       <c r="I3" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2440,49 +2449,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A1" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
+      <c r="A1" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1">
@@ -2490,36 +2499,36 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F3" s="4">
+      <c r="F3" s="10">
         <v>45932</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="4">
         <v>45577</v>
       </c>
       <c r="H3" s="2">
         <v>1</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -2546,49 +2555,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A1" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
+      <c r="A1" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1">
@@ -2596,16 +2605,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -2614,7 +2623,7 @@
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -2642,49 +2651,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A1" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
+      <c r="A1" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1">
@@ -2692,22 +2701,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="11">
+        <v>46296</v>
+      </c>
+      <c r="F3" s="4">
+        <v>45870</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="E3" s="5">
-        <v>46296</v>
-      </c>
-      <c r="F3" s="6">
-        <v>45870</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
@@ -2720,22 +2729,22 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="11">
+        <v>46296</v>
+      </c>
+      <c r="F4" s="4">
+        <v>45870</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="E4" s="5">
-        <v>46296</v>
-      </c>
-      <c r="F4" s="6">
-        <v>45870</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2" t="s">
@@ -2748,25 +2757,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="E5" s="5">
+      <c r="E5" s="11">
         <v>46342</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="4">
         <v>46281</v>
       </c>
       <c r="G5" s="2">
         <v>1</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>9</v>
@@ -2778,25 +2787,25 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E6" s="5">
+      <c r="E6" s="11">
         <v>46308</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="4">
         <v>46278</v>
       </c>
       <c r="G6" s="2">
         <v>1</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>9</v>
@@ -2808,25 +2817,25 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E7" s="5">
+      <c r="E7" s="11">
         <v>46308</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="4">
         <v>46278</v>
       </c>
       <c r="G7" s="2">
         <v>1</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>9</v>
@@ -2838,18 +2847,18 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E8" s="5">
+      <c r="E8" s="11">
         <v>46308</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="4">
         <v>46278</v>
       </c>
       <c r="G8" s="2">
@@ -2866,25 +2875,25 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="E9" s="5">
+      <c r="E9" s="11">
         <v>46381</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="4">
         <v>44190</v>
       </c>
       <c r="G9" s="2">
         <v>1</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>9</v>
@@ -2896,23 +2905,23 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D10" s="2"/>
-      <c r="E10" s="5">
+      <c r="E10" s="11">
         <v>46311</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="4">
         <v>46281</v>
       </c>
       <c r="G10" s="2">
         <v>3</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>9</v>
@@ -2955,45 +2964,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A1" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
+      <c r="A1" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="30" customHeight="1">
@@ -3001,18 +3010,18 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>137</v>
-      </c>
       <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3" s="4">
+        <v>32</v>
+      </c>
+      <c r="F3" s="10">
         <v>45993</v>
       </c>
       <c r="G3" s="2"/>
@@ -3024,16 +3033,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>139</v>
-      </c>
       <c r="D4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E4" s="2"/>
-      <c r="F4" s="4">
+      <c r="F4" s="10">
         <v>45723</v>
       </c>
       <c r="G4" s="2"/>
@@ -3047,18 +3056,18 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F5" s="4">
+      <c r="F5" s="10">
         <v>45737</v>
       </c>
       <c r="G5" s="2"/>
@@ -3069,7 +3078,7 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -3094,51 +3103,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+    </row>
+    <row r="2" spans="1:5" ht="30" customHeight="1">
+      <c r="A2" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-    </row>
-    <row r="2" spans="1:5" ht="30" customHeight="1">
-      <c r="A2" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="10" t="s">
+      <c r="E2" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="75" customHeight="1">
+      <c r="A3" s="5">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="75" customHeight="1">
-      <c r="A3" s="7">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="15">
+        <v>46582</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D3" s="8">
-        <v>46582</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>147</v>
-      </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="9" t="s">
-        <v>84</v>
+      <c r="A4" s="6" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed jasin date to 5/8/2026
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\email-reminder\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E2752C5-7922-4530-80F4-F48AE02C3D5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F97861B-D146-4B40-A250-428A471E88F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AV" sheetId="1" r:id="rId1"/>
@@ -1623,7 +1623,7 @@
         <v>46</v>
       </c>
       <c r="E10" s="11">
-        <v>46313</v>
+        <v>46239</v>
       </c>
       <c r="F10" s="2">
         <v>200</v>

</xml_diff>